<commit_message>
I updated the 'stop' class. And refactored to make that class work. Next will be separating all classes into specific classes inside domain folder
</commit_message>
<xml_diff>
--- a/logistics_data_multibranch.xlsx
+++ b/logistics_data_multibranch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kosbywonacott/Documents/Routing 2 System/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB648EC4-C3EF-7F4B-923B-77866FBE1CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C18EEF-B408-C64C-8D60-63A03AC128FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,9 +55,6 @@
     <t>Service_Time_Minutes</t>
   </si>
   <si>
-    <t>Profit_Per_Stop</t>
-  </si>
-  <si>
     <t>Time_Window_Start</t>
   </si>
   <si>
@@ -266,13 +263,16 @@
   </si>
   <si>
     <t>Failure_Simulation_Runs</t>
+  </si>
+  <si>
+    <t>Revenue_Per_Stop</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -285,6 +285,13 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -313,9 +320,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -643,28 +651,28 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>12</v>
       </c>
       <c r="D2">
         <v>25.771699999999999</v>
@@ -679,24 +687,24 @@
         <v>150</v>
       </c>
       <c r="H2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" t="s">
         <v>13</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>14</v>
-      </c>
-      <c r="J2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
         <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
       </c>
       <c r="D3">
         <v>25.781700000000001</v>
@@ -711,24 +719,24 @@
         <v>200</v>
       </c>
       <c r="H3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" t="s">
         <v>18</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>19</v>
-      </c>
-      <c r="J3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
         <v>21</v>
-      </c>
-      <c r="C4" t="s">
-        <v>22</v>
       </c>
       <c r="D4">
         <v>25.7517</v>
@@ -743,24 +751,24 @@
         <v>180</v>
       </c>
       <c r="H4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
         <v>24</v>
-      </c>
-      <c r="C5" t="s">
-        <v>25</v>
       </c>
       <c r="D5">
         <v>25.776700000000002</v>
@@ -775,24 +783,24 @@
         <v>220</v>
       </c>
       <c r="H5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" t="s">
         <v>26</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>27</v>
-      </c>
-      <c r="J5" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
         <v>33</v>
-      </c>
-      <c r="C6" t="s">
-        <v>34</v>
       </c>
       <c r="D6">
         <v>25.771699999999999</v>
@@ -807,24 +815,24 @@
         <v>185</v>
       </c>
       <c r="H6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" t="s">
         <v>35</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>36</v>
-      </c>
-      <c r="C7" t="s">
-        <v>37</v>
       </c>
       <c r="D7">
         <v>28.043900000000001</v>
@@ -839,24 +847,24 @@
         <v>140</v>
       </c>
       <c r="H7" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" t="s">
         <v>13</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>14</v>
-      </c>
-      <c r="J7" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
         <v>38</v>
-      </c>
-      <c r="C8" t="s">
-        <v>39</v>
       </c>
       <c r="D8">
         <v>28.053899999999999</v>
@@ -871,24 +879,24 @@
         <v>190</v>
       </c>
       <c r="H8" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" t="s">
         <v>18</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>19</v>
-      </c>
-      <c r="J8" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" t="s">
         <v>40</v>
-      </c>
-      <c r="C9" t="s">
-        <v>41</v>
       </c>
       <c r="D9">
         <v>28.023900000000001</v>
@@ -903,24 +911,24 @@
         <v>160</v>
       </c>
       <c r="H9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" t="s">
         <v>42</v>
-      </c>
-      <c r="C10" t="s">
-        <v>43</v>
       </c>
       <c r="D10">
         <v>28.0489</v>
@@ -935,24 +943,24 @@
         <v>210</v>
       </c>
       <c r="H10" t="s">
+        <v>25</v>
+      </c>
+      <c r="I10" t="s">
         <v>26</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>27</v>
-      </c>
-      <c r="J10" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" t="s">
         <v>44</v>
-      </c>
-      <c r="C11" t="s">
-        <v>45</v>
       </c>
       <c r="D11">
         <v>28.0139</v>
@@ -967,24 +975,24 @@
         <v>165</v>
       </c>
       <c r="H11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I11" t="s">
         <v>29</v>
       </c>
-      <c r="I11" t="s">
-        <v>30</v>
-      </c>
       <c r="J11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" t="s">
         <v>46</v>
-      </c>
-      <c r="C12" t="s">
-        <v>47</v>
       </c>
       <c r="D12">
         <v>28.038900000000002</v>
@@ -999,24 +1007,24 @@
         <v>200</v>
       </c>
       <c r="H12" t="s">
+        <v>30</v>
+      </c>
+      <c r="I12" t="s">
         <v>31</v>
       </c>
-      <c r="I12" t="s">
-        <v>32</v>
-      </c>
       <c r="J12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" t="s">
         <v>48</v>
-      </c>
-      <c r="C13" t="s">
-        <v>49</v>
       </c>
       <c r="D13">
         <v>28.018899999999999</v>
@@ -1031,24 +1039,24 @@
         <v>155</v>
       </c>
       <c r="H13" t="s">
+        <v>12</v>
+      </c>
+      <c r="I13" t="s">
         <v>13</v>
       </c>
-      <c r="I13" t="s">
-        <v>14</v>
-      </c>
       <c r="J13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" t="s">
         <v>50</v>
-      </c>
-      <c r="C14" t="s">
-        <v>51</v>
       </c>
       <c r="D14">
         <v>28.053899999999999</v>
@@ -1063,13 +1071,13 @@
         <v>175</v>
       </c>
       <c r="H14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1090,33 +1098,33 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C2">
         <v>2022</v>
@@ -1139,10 +1147,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C3">
         <v>2021</v>
@@ -1181,7 +1189,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>3</v>
@@ -1190,15 +1198,15 @@
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C2">
         <v>25.761700000000001</v>
@@ -1207,15 +1215,15 @@
         <v>-80.191800000000001</v>
       </c>
       <c r="E2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C3">
         <v>28.033899999999999</v>
@@ -1224,7 +1232,7 @@
         <v>-82.742099999999994</v>
       </c>
       <c r="E3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1243,15 +1251,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2">
         <v>10</v>
@@ -1259,7 +1267,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B3">
         <v>8</v>
@@ -1267,7 +1275,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B4">
         <v>18</v>
@@ -1275,7 +1283,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B5">
         <v>30</v>
@@ -1283,23 +1291,23 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" t="s">
         <v>73</v>
-      </c>
-      <c r="B6" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B8">
         <v>1000</v>

</xml_diff>